<commit_message>
var_name is the header name
</commit_message>
<xml_diff>
--- a/code/ctd_data/ctd_lookup_table_data.xlsx
+++ b/code/ctd_data/ctd_lookup_table_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zack.oyafuso\Work\GitHub\gap_products\code\ctd_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5496459-0986-454C-A428-59206A98FC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CDA8370-5A64-44B2-89BE-C366BF0DA910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="14400" windowHeight="7270" xr2:uid="{60C4621A-9269-41C1-A8ED-C4F6743386D3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{60C4621A-9269-41C1-A8ED-C4F6743386D3}"/>
   </bookViews>
   <sheets>
     <sheet name="CTD_DIRECTION_CODES" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
   <si>
     <t>Downcast</t>
   </si>
@@ -116,27 +116,6 @@
     <t>mS</t>
   </si>
   <si>
-    <t>Temperature</t>
-  </si>
-  <si>
-    <t>Salinity</t>
-  </si>
-  <si>
-    <t>Absolute Salinity</t>
-  </si>
-  <si>
-    <t>Pressure</t>
-  </si>
-  <si>
-    <t>Dissolved Oxygen</t>
-  </si>
-  <si>
-    <t>Turbidity (FTU)</t>
-  </si>
-  <si>
-    <t>Turbidity (NTU)</t>
-  </si>
-  <si>
     <t>Fluorescence</t>
   </si>
   <si>
@@ -171,6 +150,36 @@
   </si>
   <si>
     <t>Dissolved oxygen concentration in mg/ml (Garcia and Gordon, 1992)</t>
+  </si>
+  <si>
+    <t>TEMPERATURE_C</t>
+  </si>
+  <si>
+    <t>SALINITY_PSU</t>
+  </si>
+  <si>
+    <t>SALINITY_PPM</t>
+  </si>
+  <si>
+    <t>SALINITY_ABS</t>
+  </si>
+  <si>
+    <t>PRESSURE_DBAR</t>
+  </si>
+  <si>
+    <t>DOXY_MG_ML</t>
+  </si>
+  <si>
+    <t>DOXY_MMOL_L</t>
+  </si>
+  <si>
+    <t>PH</t>
+  </si>
+  <si>
+    <t>TURBIDITY_FTU</t>
+  </si>
+  <si>
+    <t>TURBIDITY_NTU</t>
   </si>
 </sst>
 </file>
@@ -658,13 +667,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -672,13 +681,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -686,13 +695,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s">
         <v>16</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -700,13 +709,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
         <v>17</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -714,13 +723,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
         <v>18</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -728,13 +737,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
         <v>19</v>
       </c>
       <c r="D7" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -742,13 +751,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
         <v>20</v>
       </c>
       <c r="D8" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -756,7 +765,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C9" t="s">
         <v>21</v>
@@ -770,13 +779,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="C10" t="s">
         <v>22</v>
       </c>
       <c r="D10" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
@@ -784,13 +793,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C11" t="s">
         <v>23</v>
       </c>
       <c r="D11" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
@@ -798,7 +807,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
@@ -806,13 +815,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C13" t="s">
         <v>24</v>
       </c>
       <c r="D13" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>